<commit_message>
update experts_merged.xlsx with latest data
</commit_message>
<xml_diff>
--- a/data/raw/experts_merged.xlsx
+++ b/data/raw/experts_merged.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jozef\Desktop\Projekt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B20A7B7-D6C8-450F-8860-471F716CFE28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B012BFA9-1567-4694-9F6D-DCF7F808064D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="566" uniqueCount="338">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="595" uniqueCount="392">
   <si>
     <t>dataset</t>
   </si>
@@ -1050,19 +1050,188 @@
   </si>
   <si>
     <t>N#Cc%16ccc(n%15c(=O)c%14cc%13c(=O)n(c%12ccc(c%11nc(c5ccc(n4c(=O)c3cc2c(=O)n(c1ccc(C#N)cc1)c(=O)c2cc3c4=O)cc5)nc(c%10ccc(n9c(=O)c8cc7c(=O)n(c6ccc(C#N)cc6)c(=O)c7cc8c9=O)cc%10)n%11)cc%12)c(=O)c%13cc%14c%15=O)cc%16</t>
+  </si>
+  <si>
+    <t>Nc%18ccc(c%17ccc%16[nH]c(c%15cc(c3nc2cc(c1ccc(N)c(N)c1)ccc2[nH]3)cc(n%11c(=O)c%12ccc%13c(=O)n(c%10cc(c6nc5cc(c4ccc(N)c(N)c4)ccc5[nH]6)cc(c9nc8cc(c7ccc(N)c(N)c7)ccc8[nH]9)c%10)c(=O)c%14ccc(c%11=O)c%12c%13%14)c%15)nc%16c%17)cc%18N</t>
+  </si>
+  <si>
+    <t>Nc%17ccc(c%16ccc%15[nH]c(c%14cc(c3nc2cc(c1ccc(N)c(N)c1)ccc2[nH]3)cc(n%13c(=O)c%12cc%11c(=O)n(c%10cc(c6nc5ccc(c4ccc(N)c(N)c4)cc5[nH]6)cc(c9nc8ccc(c7ccc(N)c(N)c7)cc8[nH]9)c%10)c(=O)c%11cc%12c%13=O)c%14)nc%15c%16)cc%17N</t>
+  </si>
+  <si>
+    <t>Nc7cc6nc5c2nc1cc(N)c(N)cc1nc2c4nc3cc(N)c(N)cc3nc4c5nc6cc7N</t>
+  </si>
+  <si>
+    <t>NC2=C(N)C(=O)C1N=c6c(=NC1C2=O)c4=NC3C(=O)C(N)=C(N)C(=O)C3N=c4c7=NC5C(=O)C(N)=C(N)C(=O)C5N=c67</t>
+  </si>
+  <si>
+    <t>BrC%20=CC%19Sc%18cc(Br)c(c%17ccc(c%16ccc(C(c5ccc(c4ccc(c3cc2SC1C=C(Br)C(Br)=CC1Sc2cc3Br)cc4)cc5)C(c%10ccc(c9ccc(c8cc7SC6C=C(Br)C(Br)=CC6Sc7cc8Br)cc9)cc%10)c%15ccc(c%14ccc(c%13cc%12sc%11cc(Br)c(Br)cc%11sc%12cc%13Br)cc%14)cc%15)cc%16)cc%17)cc%18SC%19C=C%20Br</t>
+  </si>
+  <si>
+    <t>BrC%20=CC%19Sc%18cc(c%17ccc(c%16ccc(C(c5ccc(c4ccc(c3ccc2SC1C=CC(Br)=CC1Sc2c3)cc4)cc5)C(c%10ccc(c9ccc(c8ccc7SC6C=CC(Br)=CC6Sc7c8)cc9)cc%10)c%15ccc(c%14ccc(c%13ccc%12sc%11ccc(Br)cc%11sc%12c%13)cc%14)cc%15)cc%16)cc%17)ccc%18SC%19C=C%20</t>
+  </si>
+  <si>
+    <t>Brak symetrycznej struktury</t>
+  </si>
+  <si>
+    <t>C#Cc%23ccc(N%22COc%21cc%20CN(C#Cc%19ccc%18CN(c%17ccc(N(c8ccc(N7COc6cc(C#Cc5ccc(N4COc3cc2CN(c1ccc(C#C)cc1)COc2cc3C4)cc5)ccc6C7)cc8)c%16ccc(N%15COc%14cc(C#Cc%13ccc(N%12COc%11cc%10CN(c9ccc(C#C)cc9)COc%10cc%11C%12)cc%13)ccc%14C%15)cc%16)cc%17)COc%18c%19)COc%20cc%21C%22)cc%23</t>
+  </si>
+  <si>
+    <t>CCc%15ccc(NCc%14cc(O)c(CNc%13ccc(CCc%12ccc(CNc%11ccc(N(c5ccc(NCc4ccc(CCc3ccc(NCc2cc(O)c(CNc1ccc(CC)cc1)cc2O)cc3)cc4O)cc5)c%10ccc(NCc9ccc(CCc8ccc(NCc7cc(O)c(CNc6ccc(CC)cc6)cc7O)cc8)cc9O)cc%10)cc%11)c(O)c%12)cc%13)cc%14O)cc%15</t>
+  </si>
+  <si>
+    <t>COc7ccc(C(c1ccc(OC)cc1)=c5c2ccccc2c(=C(c3ccc(OC)cc3)c4ccc(OC)cc4)c6ccccc56)cc7</t>
+  </si>
+  <si>
+    <t>Clc%11nc(Cl)nc(c%10ccc(C(c2ccc(c1nc(Cl)nc(Cl)n1)cc2)=c8c3ccccc3c(=C(c5ccc(c4nc(Cl)nc(Cl)n4)cc5)c7ccc(c6nc(Cl)nc(Cl)n6)cc7)c9ccccc89)cc%10)n%11</t>
+  </si>
+  <si>
+    <t>O=Cc4ccc(/C=N/c3nc(/N=C/c1ccc(C=O)cc1)nc(/N=C/c2ccc(C=O)cc2)n3)cc4</t>
+  </si>
+  <si>
+    <t>O=Cc4ccc(/C=N/c3ccc(Oc2ccc(/N=C/c1ccc(C=O)cc1)cc2)cc3)cc4</t>
+  </si>
+  <si>
+    <t>c7ncnc(c6ccc(c5cc(c2ccc(c1ncncn1)cc2)nc(c4ccc(c3ncncn3)cc4)c5)cc6)n7</t>
+  </si>
+  <si>
+    <t>O=Cc7c(O)c(C=O)c(=O)c(=CNc6ccc(c5cc(c2ccc(NC=c1c(O)c(C=O)c(O)c(C=O)c1=O)cc2)nc(c4ccc(NC=c3c(O)c(C=O)c(O)c(C=O)c3=O)cc4)c5)cc6)c7O</t>
+  </si>
+  <si>
+    <t>O=Cc6c(O)c(C=O)c(=O)c(=CNc5ccc(N(c2ccc(NC=c1c(O)c(C=O)c(O)c(C=O)c1=O)cc2)c4ccc(NC=c3c(O)c(C=O)c(O)c(C=O)c3=O)cc4)cc5)c6O</t>
+  </si>
+  <si>
+    <t>O=Cc7c(O)c(C=O)c(=O)c(=CNc6ccc(n5c2ccc(NC=c1c(O)c(C=O)c(O)c(C=O)c1=O)cc2c4cc(NC=c3c(O)c(C=O)c(O)c(C=O)c3=O)ccc45)cc6)c7O</t>
+  </si>
+  <si>
+    <t>O=Cc%12ccc(N(c1ccc(C=O)cc1)c%11ccc(/C=N/c%10ccc(N(c5ccc(/N=C/c4ccc(N(c2ccc(C=O)cc2)c3ccc(C=O)cc3)cc4)cc5)c9ccc(/N=C/c8ccc(N(c6ccc(C=O)cc6)c7ccc(C=O)cc7)cc8)cc9)cc%10)cc%11)cc%12</t>
+  </si>
+  <si>
+    <t>O=Cc%15ccc(c%14cc(c1ccc(C=O)cc1)nc(c%13ccc(/C=N/c%12ccc(N(c6ccc(/N=C/c5ccc(c4cc(c2ccc(C=O)cc2)cc(c3ccc(C=O)cc3)n4)cc5)cc6)c%11ccc(/N=C/c%10ccc(c9cc(c7ccc(C=O)cc7)cc(c8ccc(C=O)cc8)n9)cc%10)cc%11)cc%12)cc%13)c%14)cc%15</t>
+  </si>
+  <si>
+    <t>O=Cc%15ccc(c%14nc(c1ccc(C=O)cc1)nc(c%13ccc(/C=N/c%12ccc(N(c6ccc(/N=C/c5ccc(c4nc(c2ccc(C=O)cc2)nc(c3ccc(C=O)cc3)n4)cc5)cc6)c%11ccc(/N=C/c%10ccc(c9nc(c7ccc(C=O)cc7)nc(c8ccc(C=O)cc8)n9)cc%10)cc%11)cc%12)cc%13)n%14)cc%15</t>
+  </si>
+  <si>
+    <t>O=N(=O)c%13ccc([n+]%12ccc(c%11cc[n+](c%10ccc(c9cc(c4ccc([n+]3ccc(c2cc[n+](c1ccc(N(=O)=O)cc1N(=O)=O)cc2)cc3)cc4)cc(c8ccc([n+]7ccc(c6cc[n+](c5ccc(N(=O)=O)cc5N(=O)=O)cc6)cc7)cc8)c9)cc%10)cc%11)cc%12)c(N(=O)=O)c%13</t>
+  </si>
+  <si>
+    <t>O=Cc%13ccc(N(c1ccc(C=O)cc1)c%12ccc(/C=N/c%11ccc(c%10nc(c5ccc(/N=C/c4ccc(N(c2ccc(C=O)cc2)c3ccc(C=O)cc3)cc4)cc5)nc(c9ccc(/N=C/c8ccc(N(c6ccc(C=O)cc6)c7ccc(C=O)cc7)cc8)cc9)n%10)cc%11)cc%12)cc%13</t>
+  </si>
+  <si>
+    <t>O=Cc%13ccc(N(c1ccc(C=O)cc1)c%12ccc(/C=N/c%11ccc(n%10c5ccc(/N=C/c4ccc(N(c2ccc(C=O)cc2)c3ccc(C=O)cc3)cc4)cc5c9cc(/N=C/c8ccc(N(c6ccc(C=O)cc6)c7ccc(C=O)cc7)cc8)ccc9%10)cc%11)cc%12)cc%13</t>
+  </si>
+  <si>
+    <t>O=Cc%16ccc(c%15cc(c1ccc(C=O)cc1)nc(c%14ccc(/C=N/c%13ccc(c%12nc(c6ccc(/N=C/c5ccc(c4cc(c2ccc(C=O)cc2)cc(c3ccc(C=O)cc3)n4)cc5)cc6)nc(c%11ccc(/N=C/c%10ccc(c9cc(c7ccc(C=O)cc7)cc(c8ccc(C=O)cc8)n9)cc%10)cc%11)n%12)cc%13)cc%14)c%15)cc%16</t>
+  </si>
+  <si>
+    <t>O=Cc%16ccc(c%15nc(c1ccc(C=O)cc1)nc(c%14ccc(/C=N/c%13ccc(c%12nc(c6ccc(/N=C/c5ccc(c4nc(c2ccc(C=O)cc2)nc(c3ccc(C=O)cc3)n4)cc5)cc6)nc(c%11ccc(/N=C/c%10ccc(c9nc(c7ccc(C=O)cc7)nc(c8ccc(C=O)cc8)n9)cc%10)cc%11)n%12)cc%13)cc%14)n%15)cc%16</t>
+  </si>
+  <si>
+    <t>O=Cc%16ccc(c%15cc(c1ccc(C=O)cc1)nc(c%14ccc(/C=N/c%13ccc(n%12c6ccc(/N=C/c5ccc(c4cc(c2ccc(C=O)cc2)cc(c3ccc(C=O)cc3)n4)cc5)cc6c%11cc(/N=C/c%10ccc(c9cc(c7ccc(C=O)cc7)cc(c8ccc(C=O)cc8)n9)cc%10)ccc%11%12)cc%13)cc%14)c%15)cc%16</t>
+  </si>
+  <si>
+    <t>O=Cc%16ccc(c%15nc(c1ccc(C=O)cc1)nc(c%14ccc(/C=N/c%13ccc(n%12c6ccc(/N=C/c5ccc(c4nc(c2ccc(C=O)cc2)nc(c3ccc(C=O)cc3)n4)cc5)cc6c%11cc(/N=C/c%10ccc(c9nc(c7ccc(C=O)cc7)nc(c8ccc(C=O)cc8)n9)cc%10)ccc%11%12)cc%13)cc%14)n%15)cc%16</t>
+  </si>
+  <si>
+    <t>O=C8c7cc(n3c1ccccc1c2ccccc23)c(n6c4ccccc4c5ccccc56)cc7C(=O)C8c%17cc(n%16c(=O)c%15cc(n%11c9ccccc9c%10ccccc%10%11)c(n%14c%12ccccc%12c%13ccccc%13%14)cc%15c%16=O)c(O)cc%17O</t>
+  </si>
+  <si>
+    <t>O=S%20(=O)c1ccc(Br)cc1S(=O)(=O)c%19cc(c%18ccc(c%17ccc(C(c6ccc(c5ccc(c2ccc4c(c2)S(=O)(=O)C3C=CC(Br)=CC3S4(=O)=O)cc5)cc6)C(c%11ccc(c%10ccc(c7ccc9c(c7)S(=O)(=O)C8C=CC(Br)=CC8S9(=O)=O)cc%10)cc%11)c%16ccc(c%15ccc(c%12ccc%14c(c%12)S(=O)(=O)C%13C=C(Br)C=CC%13S%14(=O)=O)cc%15)cc%16)cc%17)cc%18)ccc%19%20</t>
+  </si>
+  <si>
+    <t>Brc1ccc%39c(c1)c2cc(Br)ccc2c%40nc%38cc%37nc%36c%34ccc(c%30cc(c3ccc%10c(c3)c4ccccc4c%11nc9cc8nc7c5ccc(Br)cc5c6cc(Br)ccc6c7nc8cc9nc%10%11)c%31ccc%33c(c%12ccc%19c(c%12)c%13ccccc%13c%20nc%18cc%17nc%16c%14ccc(Br)cc%14c%15cc(Br)ccc%15c%16nc%17cc%18nc%19%20)cc(c%21ccc%28c(c%21)c%22ccccc%22c%29nc%27cc%26nc%25c%23ccc(Br)cc%23c%24cc(Br)ccc%24c%25nc%26cc%27nc%28%29)c%32CCc%30c%31c%32%33)cc%34c%35ccccc%35c%36nc%37cc%38nc%39%40</t>
+  </si>
+  <si>
+    <t>Brc1ccc%31c(c1)c%24cc(c%23ccc(c%22cc(c%11ccc(c2ccc9c(c2)c3cc(Br)ccc3c%10nc8cc7nc6c4ccc(Br)cc4c5cc(Br)ccc5c6nc7cc8nc9%10)cc%11)cc(c%21ccc(c%12ccc%19c(c%12)c%13cc(Br)ccc%13c%20nc%18cc%17nc%16c%14ccc(Br)cc%14c%15cc(Br)ccc%15c%16nc%17cc%18nc%19%20)cc%21)n%22)cc%23)ccc%24c%32cc%30nc%29cc%28nc%27c%25ccc(Br)cc%25c%26cc(Br)ccc%26c%27nc%28cc%29nc%30cc%31%32</t>
+  </si>
+  <si>
+    <t>Brc1ccc%31c(c1)c%24cc(c%23ccc(c%22nc(c%11ccc(c2ccc9c(c2)c3cc(Br)ccc3c%10nc8cc7nc6c4ccc(Br)cc4c5cc(Br)ccc5c6nc7cc8nc9%10)cc%11)nc(c%21ccc(c%12ccc%19c(c%12)c%13cc(Br)ccc%13c%20nc%18cc%17nc%16c%14ccc(Br)cc%14c%15cc(Br)ccc%15c%16nc%17cc%18nc%19%20)cc%21)n%22)cc%23)ccc%24c%32cc%30nc%29cc%28nc%27c%25ccc(Br)cc%25c%26cc(Br)ccc%26c%27nc%28cc%29nc%30cc%31%32</t>
+  </si>
+  <si>
+    <t>KOBALT !</t>
+  </si>
+  <si>
+    <t>Nie mogę znalezć,dziwna struktura</t>
+  </si>
+  <si>
+    <t>MOLIBDEN !</t>
+  </si>
+  <si>
+    <t>Rodnik</t>
+  </si>
+  <si>
+    <t>Cc1nc(C)nc(C)n1</t>
+  </si>
+  <si>
+    <t>?????</t>
+  </si>
+  <si>
+    <t>Komentarz</t>
+  </si>
+  <si>
+    <t>Miało być bez metali</t>
+  </si>
+  <si>
+    <t>Sferyczna struktura , wygląda jak glukoza</t>
+  </si>
+  <si>
+    <t>Tutaj kolejny cukier, podobne do izomaltozy</t>
+  </si>
+  <si>
+    <t>Potrzebne są mi substraty by zobaczyć co powstanie</t>
+  </si>
+  <si>
+    <t>nie wiem co to, nie mogę załadować SMILESA</t>
+  </si>
+  <si>
+    <t>Mozliwe ,ale brak koncówek, potrzebne substraty</t>
+  </si>
+  <si>
+    <t>Dziwny zwiazek, potrzebuję DOI by stwierdzić czy coś z tego będzie</t>
+  </si>
+  <si>
+    <t>Nc4ccc(C(c1ccc(N)cc1)(c2ccc(N)cc2)c3ccc(N)cc3)cc4</t>
+  </si>
+  <si>
+    <t>Sama anilina ,mało prawdopodobne...</t>
+  </si>
+  <si>
+    <t>N#Cc%13ccc(c%11nn(c%10ccc(c9nc(c4ccc(n3nc(c1ccc(C#N)cc1)c2ccccc2c3=O)cc4)nc(c8ccc(n7nc(c5ccc(C#N)cc5)c6ccccc6c7=O)cc8)n9)cc%10)c(=O)c%12ccccc%11%12)cc%13</t>
+  </si>
+  <si>
+    <t>Magnez</t>
+  </si>
+  <si>
+    <t>Cynk</t>
+  </si>
+  <si>
+    <t>Brak</t>
+  </si>
+  <si>
+    <t>Mozliwe ,ale brakuje substratów</t>
+  </si>
+  <si>
+    <t>????</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="238"/>
     </font>
   </fonts>
   <fills count="4">
@@ -1085,7 +1254,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1093,11 +1262,26 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1115,6 +1299,16 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -6352,7 +6546,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F113"/>
+  <dimension ref="A1:G113"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.28515625" style="1" customWidth="1"/>
@@ -6361,9 +6555,10 @@
     <col min="4" max="4" width="50.7109375" style="1" customWidth="1"/>
     <col min="5" max="5" width="14.5703125" style="1" customWidth="1"/>
     <col min="6" max="6" width="23.140625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="13.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -6382,8 +6577,11 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G1" s="1" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="300" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
@@ -6400,7 +6598,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" ht="300" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
@@ -6417,7 +6615,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" ht="300" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
@@ -6434,7 +6632,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="5" spans="1:6" s="6" customFormat="1" ht="300" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" s="6" customFormat="1" ht="300" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>6</v>
       </c>
@@ -6452,7 +6650,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" ht="300" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
@@ -6469,7 +6667,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="7" spans="1:6" s="6" customFormat="1" ht="300" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" s="6" customFormat="1" ht="300" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>6</v>
       </c>
@@ -6487,7 +6685,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" ht="300" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>6</v>
       </c>
@@ -6504,7 +6702,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" ht="300" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>6</v>
       </c>
@@ -6521,7 +6719,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" ht="300" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>6</v>
       </c>
@@ -6538,7 +6736,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" ht="300" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>6</v>
       </c>
@@ -6555,7 +6753,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" ht="300" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>6</v>
       </c>
@@ -6572,7 +6770,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" ht="300" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>6</v>
       </c>
@@ -6589,7 +6787,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" ht="300" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>6</v>
       </c>
@@ -6606,7 +6804,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" ht="300" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>6</v>
       </c>
@@ -6623,7 +6821,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" ht="300" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>6</v>
       </c>
@@ -6857,8 +7055,8 @@
       <c r="E29" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="F29" s="1" t="s">
-        <v>10</v>
+      <c r="F29" s="7" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
@@ -6874,8 +7072,8 @@
       <c r="E30" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="F30" s="1" t="s">
-        <v>10</v>
+      <c r="F30" s="2" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="31" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
@@ -6891,24 +7089,25 @@
       <c r="E31" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="F31" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="1" t="s">
+      <c r="F31" s="2" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" s="6" customFormat="1" ht="300" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="B32" s="2" t="s">
+      <c r="B32" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="C32" s="2" t="s">
+      <c r="C32" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="E32" s="1" t="s">
+      <c r="D32" s="4"/>
+      <c r="E32" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="F32" s="1" t="s">
+      <c r="F32" s="4" t="s">
         <v>10</v>
       </c>
     </row>
@@ -6926,7 +7125,7 @@
         <v>80</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>10</v>
+        <v>335</v>
       </c>
     </row>
     <row r="34" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
@@ -6942,8 +7141,8 @@
       <c r="E34" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="F34" s="1" t="s">
-        <v>10</v>
+      <c r="F34" s="2" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="35" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
@@ -6959,8 +7158,8 @@
       <c r="E35" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="F35" s="1" t="s">
-        <v>10</v>
+      <c r="F35" s="2" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="36" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
@@ -6977,7 +7176,7 @@
         <v>105</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>10</v>
+        <v>338</v>
       </c>
     </row>
     <row r="37" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
@@ -6993,8 +7192,8 @@
       <c r="E37" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="F37" s="1" t="s">
-        <v>10</v>
+      <c r="F37" s="2" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="38" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
@@ -7010,8 +7209,8 @@
       <c r="E38" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="F38" s="1" t="s">
-        <v>10</v>
+      <c r="F38" s="7" t="s">
+        <v>339</v>
       </c>
     </row>
     <row r="39" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
@@ -7027,8 +7226,8 @@
       <c r="E39" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="F39" s="1" t="s">
-        <v>10</v>
+      <c r="F39" s="2" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="40" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
@@ -7044,8 +7243,8 @@
       <c r="E40" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F40" s="1" t="s">
-        <v>10</v>
+      <c r="F40" s="2" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="41" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
@@ -7061,8 +7260,8 @@
       <c r="E41" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="F41" s="1" t="s">
-        <v>10</v>
+      <c r="F41" s="2" t="s">
+        <v>118</v>
       </c>
     </row>
     <row r="42" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
@@ -7078,8 +7277,8 @@
       <c r="E42" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="F42" s="1" t="s">
-        <v>10</v>
+      <c r="F42" s="2" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="43" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
@@ -7096,7 +7295,7 @@
         <v>126</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>10</v>
+        <v>340</v>
       </c>
     </row>
     <row r="44" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
@@ -7113,7 +7312,7 @@
         <v>129</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>10</v>
+        <v>341</v>
       </c>
     </row>
     <row r="45" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
@@ -7129,8 +7328,8 @@
       <c r="E45" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="F45" s="1" t="s">
-        <v>10</v>
+      <c r="F45" s="2" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="46" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
@@ -7146,8 +7345,8 @@
       <c r="E46" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="F46" s="1" t="s">
-        <v>10</v>
+      <c r="F46" s="2" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="47" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
@@ -7163,8 +7362,8 @@
       <c r="E47" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="F47" s="1" t="s">
-        <v>10</v>
+      <c r="F47" s="8" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="48" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
@@ -7181,7 +7380,7 @@
         <v>77</v>
       </c>
       <c r="F48" s="1" t="s">
-        <v>10</v>
+        <v>334</v>
       </c>
     </row>
     <row r="49" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
@@ -7197,8 +7396,8 @@
       <c r="E49" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="F49" s="1" t="s">
-        <v>10</v>
+      <c r="F49" s="2" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="50" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
@@ -7214,8 +7413,8 @@
       <c r="E50" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="F50" s="1" t="s">
-        <v>10</v>
+      <c r="F50" s="2" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="51" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
@@ -7232,7 +7431,7 @@
         <v>145</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>10</v>
+        <v>342</v>
       </c>
     </row>
     <row r="52" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
@@ -7249,7 +7448,7 @@
         <v>148</v>
       </c>
       <c r="F52" s="1" t="s">
-        <v>10</v>
+        <v>343</v>
       </c>
     </row>
     <row r="53" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
@@ -7266,24 +7465,25 @@
         <v>151</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="54" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="1" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" s="10" customFormat="1" ht="300" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A54" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="B54" s="2" t="s">
+      <c r="B54" s="9" t="s">
         <v>152</v>
       </c>
-      <c r="C54" s="2" t="s">
+      <c r="C54" s="9" t="s">
         <v>153</v>
       </c>
-      <c r="E54" s="1" t="s">
+      <c r="D54" s="3"/>
+      <c r="E54" s="3" t="s">
         <v>154</v>
       </c>
-      <c r="F54" s="1" t="s">
-        <v>10</v>
+      <c r="F54" s="3" t="s">
+        <v>344</v>
       </c>
     </row>
     <row r="55" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
@@ -7300,7 +7500,7 @@
         <v>157</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>10</v>
+        <v>346</v>
       </c>
     </row>
     <row r="56" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
@@ -7317,7 +7517,7 @@
         <v>160</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>10</v>
+        <v>347</v>
       </c>
     </row>
     <row r="57" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
@@ -7334,7 +7534,7 @@
         <v>163</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>10</v>
+        <v>348</v>
       </c>
     </row>
     <row r="58" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
@@ -7350,8 +7550,8 @@
       <c r="E58" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="F58" s="1" t="s">
-        <v>10</v>
+      <c r="F58" s="2" t="s">
+        <v>351</v>
       </c>
     </row>
     <row r="59" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
@@ -7368,24 +7568,25 @@
         <v>168</v>
       </c>
       <c r="F59" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="60" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="1" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" s="10" customFormat="1" ht="300" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A60" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="B60" s="2" t="s">
+      <c r="B60" s="9" t="s">
         <v>169</v>
       </c>
-      <c r="C60" s="2" t="s">
+      <c r="C60" s="9" t="s">
         <v>170</v>
       </c>
-      <c r="E60" s="1" t="s">
+      <c r="D60" s="3"/>
+      <c r="E60" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="F60" s="1" t="s">
-        <v>10</v>
+      <c r="F60" s="3" t="s">
+        <v>350</v>
       </c>
     </row>
     <row r="61" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
@@ -7402,7 +7603,7 @@
         <v>174</v>
       </c>
       <c r="F61" s="1" t="s">
-        <v>10</v>
+        <v>353</v>
       </c>
     </row>
     <row r="62" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
@@ -7419,7 +7620,7 @@
         <v>177</v>
       </c>
       <c r="F62" s="1" t="s">
-        <v>10</v>
+        <v>352</v>
       </c>
     </row>
     <row r="63" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
@@ -7436,7 +7637,7 @@
         <v>180</v>
       </c>
       <c r="F63" s="1" t="s">
-        <v>10</v>
+        <v>354</v>
       </c>
     </row>
     <row r="64" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
@@ -7453,7 +7654,7 @@
         <v>183</v>
       </c>
       <c r="F64" s="1" t="s">
-        <v>10</v>
+        <v>355</v>
       </c>
     </row>
     <row r="65" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
@@ -7470,7 +7671,7 @@
         <v>186</v>
       </c>
       <c r="F65" s="1" t="s">
-        <v>10</v>
+        <v>356</v>
       </c>
     </row>
     <row r="66" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
@@ -7487,7 +7688,7 @@
         <v>189</v>
       </c>
       <c r="F66" s="1" t="s">
-        <v>10</v>
+        <v>357</v>
       </c>
     </row>
     <row r="67" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
@@ -7504,7 +7705,7 @@
         <v>36</v>
       </c>
       <c r="F67" s="1" t="s">
-        <v>10</v>
+        <v>358</v>
       </c>
     </row>
     <row r="68" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
@@ -7521,7 +7722,7 @@
         <v>194</v>
       </c>
       <c r="F68" s="1" t="s">
-        <v>10</v>
+        <v>359</v>
       </c>
     </row>
     <row r="69" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
@@ -7538,7 +7739,7 @@
         <v>197</v>
       </c>
       <c r="F69" s="1" t="s">
-        <v>10</v>
+        <v>360</v>
       </c>
     </row>
     <row r="70" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
@@ -7555,7 +7756,7 @@
         <v>200</v>
       </c>
       <c r="F70" s="1" t="s">
-        <v>10</v>
+        <v>361</v>
       </c>
     </row>
     <row r="71" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
@@ -7572,7 +7773,7 @@
         <v>200</v>
       </c>
       <c r="F71" s="1" t="s">
-        <v>10</v>
+        <v>362</v>
       </c>
     </row>
     <row r="72" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
@@ -7589,7 +7790,7 @@
         <v>205</v>
       </c>
       <c r="F72" s="1" t="s">
-        <v>10</v>
+        <v>363</v>
       </c>
     </row>
     <row r="73" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
@@ -7606,7 +7807,7 @@
         <v>208</v>
       </c>
       <c r="F73" s="1" t="s">
-        <v>10</v>
+        <v>364</v>
       </c>
     </row>
     <row r="74" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
@@ -7623,7 +7824,7 @@
         <v>211</v>
       </c>
       <c r="F74" s="1" t="s">
-        <v>10</v>
+        <v>365</v>
       </c>
     </row>
     <row r="75" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
@@ -7640,7 +7841,7 @@
         <v>214</v>
       </c>
       <c r="F75" s="1" t="s">
-        <v>10</v>
+        <v>366</v>
       </c>
     </row>
     <row r="76" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
@@ -7657,7 +7858,7 @@
         <v>217</v>
       </c>
       <c r="F76" s="1" t="s">
-        <v>10</v>
+        <v>367</v>
       </c>
     </row>
     <row r="77" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
@@ -7674,7 +7875,7 @@
         <v>220</v>
       </c>
       <c r="F77" s="1" t="s">
-        <v>10</v>
+        <v>368</v>
       </c>
     </row>
     <row r="78" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
@@ -7691,7 +7892,7 @@
         <v>223</v>
       </c>
       <c r="F78" s="1" t="s">
-        <v>10</v>
+        <v>369</v>
       </c>
     </row>
     <row r="79" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
@@ -7707,8 +7908,8 @@
       <c r="E79" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="F79" s="1" t="s">
-        <v>10</v>
+      <c r="F79" s="2" t="s">
+        <v>224</v>
       </c>
     </row>
     <row r="80" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
@@ -7725,10 +7926,10 @@
         <v>230</v>
       </c>
       <c r="F80" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="81" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" ht="300" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="1" t="s">
         <v>227</v>
       </c>
@@ -7741,11 +7942,14 @@
       <c r="E81" s="1" t="s">
         <v>232</v>
       </c>
-      <c r="F81" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="82" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F81" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G81" s="1" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="82" spans="1:7" ht="300" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="1" t="s">
         <v>227</v>
       </c>
@@ -7759,10 +7963,13 @@
         <v>235</v>
       </c>
       <c r="F82" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="83" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
+        <v>372</v>
+      </c>
+      <c r="G82" s="1" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7" ht="300" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="1" t="s">
         <v>236</v>
       </c>
@@ -7775,11 +7982,14 @@
       <c r="E83" s="1" t="s">
         <v>239</v>
       </c>
-      <c r="F83" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="84" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F83" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="G83" s="2" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="84" spans="1:7" ht="300" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="1" t="s">
         <v>236</v>
       </c>
@@ -7792,11 +8002,14 @@
       <c r="E84" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="F84" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="85" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F84" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="G84" s="2" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="85" spans="1:7" ht="300" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="1" t="s">
         <v>236</v>
       </c>
@@ -7810,10 +8023,13 @@
         <v>25</v>
       </c>
       <c r="F85" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="86" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
+        <v>373</v>
+      </c>
+      <c r="G85" s="1" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="86" spans="1:7" ht="300" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="1" t="s">
         <v>236</v>
       </c>
@@ -7826,11 +8042,14 @@
       <c r="E86" s="1" t="s">
         <v>246</v>
       </c>
-      <c r="F86" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="87" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F86" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G86" s="1" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="87" spans="1:7" ht="300" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87" s="1" t="s">
         <v>236</v>
       </c>
@@ -7843,11 +8062,14 @@
       <c r="E87" s="1" t="s">
         <v>248</v>
       </c>
-      <c r="F87" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="88" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F87" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G87" s="1" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="88" spans="1:7" ht="300" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="1" t="s">
         <v>236</v>
       </c>
@@ -7860,11 +8082,14 @@
       <c r="E88" s="1" t="s">
         <v>251</v>
       </c>
-      <c r="F88" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="89" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F88" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="G88" s="1" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="89" spans="1:7" ht="300" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A89" s="1" t="s">
         <v>236</v>
       </c>
@@ -7877,11 +8102,14 @@
       <c r="E89" s="1" t="s">
         <v>254</v>
       </c>
-      <c r="F89" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="90" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F89" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="G89" s="1" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="90" spans="1:7" ht="300" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A90" s="1" t="s">
         <v>236</v>
       </c>
@@ -7894,11 +8122,14 @@
       <c r="E90" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="F90" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="91" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F90" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="G90" s="1" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="91" spans="1:7" ht="300" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A91" s="1" t="s">
         <v>236</v>
       </c>
@@ -7912,10 +8143,11 @@
         <v>259</v>
       </c>
       <c r="F91" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="92" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
+        <v>374</v>
+      </c>
+      <c r="G91" s="1"/>
+    </row>
+    <row r="92" spans="1:7" ht="300" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A92" s="1" t="s">
         <v>236</v>
       </c>
@@ -7928,11 +8160,14 @@
       <c r="E92" s="1" t="s">
         <v>261</v>
       </c>
-      <c r="F92" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="93" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F92" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G92" s="1" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="93" spans="1:7" ht="300" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A93" s="1" t="s">
         <v>236</v>
       </c>
@@ -7946,10 +8181,13 @@
         <v>264</v>
       </c>
       <c r="F93" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="94" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
+        <v>375</v>
+      </c>
+      <c r="G93" s="1" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="94" spans="1:7" ht="300" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="1" t="s">
         <v>236</v>
       </c>
@@ -7963,10 +8201,13 @@
         <v>25</v>
       </c>
       <c r="F94" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="95" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
+        <v>375</v>
+      </c>
+      <c r="G94" s="1" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="95" spans="1:7" ht="300" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A95" s="1" t="s">
         <v>236</v>
       </c>
@@ -7980,10 +8221,13 @@
         <v>269</v>
       </c>
       <c r="F95" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="96" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
+        <v>375</v>
+      </c>
+      <c r="G95" s="1" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="96" spans="1:7" ht="300" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A96" s="1" t="s">
         <v>236</v>
       </c>
@@ -7997,10 +8241,13 @@
         <v>272</v>
       </c>
       <c r="F96" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="97" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
+        <v>375</v>
+      </c>
+      <c r="G96" s="1" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="97" spans="1:7" ht="300" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A97" s="1" t="s">
         <v>236</v>
       </c>
@@ -8014,10 +8261,13 @@
         <v>25</v>
       </c>
       <c r="F97" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="98" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
+        <v>375</v>
+      </c>
+      <c r="G97" s="1" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="98" spans="1:7" ht="300" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A98" s="1" t="s">
         <v>236</v>
       </c>
@@ -8031,10 +8281,13 @@
         <v>277</v>
       </c>
       <c r="F98" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="99" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
+        <v>375</v>
+      </c>
+      <c r="G98" s="1" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="99" spans="1:7" ht="300" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A99" s="1" t="s">
         <v>236</v>
       </c>
@@ -8048,10 +8301,13 @@
         <v>280</v>
       </c>
       <c r="F99" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="100" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
+        <v>375</v>
+      </c>
+      <c r="G99" s="1" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="100" spans="1:7" ht="300" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A100" s="1" t="s">
         <v>236</v>
       </c>
@@ -8065,10 +8321,13 @@
         <v>283</v>
       </c>
       <c r="F100" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="101" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
+        <v>384</v>
+      </c>
+      <c r="G100" s="1" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="101" spans="1:7" ht="300" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A101" s="1" t="s">
         <v>236</v>
       </c>
@@ -8082,10 +8341,10 @@
         <v>286</v>
       </c>
       <c r="F101" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="102" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="102" spans="1:7" ht="300" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A102" s="1" t="s">
         <v>236</v>
       </c>
@@ -8098,11 +8357,14 @@
       <c r="E102" s="1" t="s">
         <v>261</v>
       </c>
-      <c r="F102" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="103" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F102" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G102" s="1" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="103" spans="1:7" ht="300" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="1" t="s">
         <v>236</v>
       </c>
@@ -8116,10 +8378,13 @@
         <v>290</v>
       </c>
       <c r="F103" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="104" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
+        <v>391</v>
+      </c>
+      <c r="G103" s="1" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="104" spans="1:7" ht="300" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A104" s="1" t="s">
         <v>236</v>
       </c>
@@ -8133,10 +8398,10 @@
         <v>232</v>
       </c>
       <c r="F104" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="105" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="105" spans="1:7" ht="300" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A105" s="1" t="s">
         <v>236</v>
       </c>
@@ -8149,11 +8414,14 @@
       <c r="E105" s="1" t="s">
         <v>294</v>
       </c>
-      <c r="F105" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="106" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F105" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G105" s="1" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="106" spans="1:7" ht="300" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A106" s="1" t="s">
         <v>236</v>
       </c>
@@ -8166,11 +8434,14 @@
       <c r="E106" s="1" t="s">
         <v>296</v>
       </c>
-      <c r="F106" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="107" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F106" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G106" s="1" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="107" spans="1:7" ht="300" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A107" s="1" t="s">
         <v>236</v>
       </c>
@@ -8184,10 +8455,10 @@
         <v>299</v>
       </c>
       <c r="F107" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="108" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="108" spans="1:7" ht="300" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A108" s="1" t="s">
         <v>236</v>
       </c>
@@ -8201,10 +8472,13 @@
         <v>302</v>
       </c>
       <c r="F108" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="109" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
+        <v>391</v>
+      </c>
+      <c r="G108" s="1" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="109" spans="1:7" ht="300" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A109" s="1" t="s">
         <v>236</v>
       </c>
@@ -8218,10 +8492,10 @@
         <v>305</v>
       </c>
       <c r="F109" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="110" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="110" spans="1:7" ht="300" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A110" s="1" t="s">
         <v>236</v>
       </c>
@@ -8235,10 +8509,13 @@
         <v>308</v>
       </c>
       <c r="F110" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="111" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
+        <v>389</v>
+      </c>
+      <c r="G110" s="1" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="111" spans="1:7" ht="300" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A111" s="1" t="s">
         <v>236</v>
       </c>
@@ -8252,10 +8529,13 @@
         <v>311</v>
       </c>
       <c r="F111" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="112" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
+        <v>391</v>
+      </c>
+      <c r="G111" s="1" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="112" spans="1:7" ht="300" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A112" s="1" t="s">
         <v>236</v>
       </c>
@@ -8269,10 +8549,13 @@
         <v>314</v>
       </c>
       <c r="F112" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="113" spans="1:6" ht="300" customHeight="1" x14ac:dyDescent="0.25">
+        <v>344</v>
+      </c>
+      <c r="G112" s="1" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="113" spans="1:7" ht="300" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A113" s="1" t="s">
         <v>236</v>
       </c>
@@ -8286,7 +8569,10 @@
         <v>316</v>
       </c>
       <c r="F113" s="1" t="s">
-        <v>10</v>
+        <v>391</v>
+      </c>
+      <c r="G113" s="1" t="s">
+        <v>383</v>
       </c>
     </row>
   </sheetData>

</xml_diff>